<commit_message>
Update registration tests and add exploratory cases
</commit_message>
<xml_diff>
--- a/test-cases/exploratory-testing/exploratory-testing.xlsx
+++ b/test-cases/exploratory-testing/exploratory-testing.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
   <si>
     <t>AUTH-012</t>
   </si>
@@ -108,13 +108,34 @@
   </si>
   <si>
     <t>1. Отправить POST /authenticate/login/</t>
+  </si>
+  <si>
+    <t>REG-049</t>
+  </si>
+  <si>
+    <t>Регистрация с пустым значением invite_hash</t>
+  </si>
+  <si>
+    <t>Пользователь не зарегистрирован в системе.</t>
+  </si>
+  <si>
+    <t>Уникальный валидный email; валидный пароль; profession_id1 - валидное значение, profession_id2 - валидное значение, profession_id3 - валидное значение, "invite_hash" : ""</t>
+  </si>
+  <si>
+    <t>1. Отправить POST на /api/v1/authenticate/register/ с указанными тестовыми данными</t>
+  </si>
+  <si>
+    <t>Ожидаемое поведение не определено требованиями.</t>
+  </si>
+  <si>
+    <t>Сервер возвращает HTTP 201 Created. Регистрация успешно завершается при передаче пустой строки в поле invite_hash.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,6 +153,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -196,12 +223,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -213,42 +237,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
+  <dxfs count="11">
     <dxf>
       <font>
         <b val="0"/>
@@ -269,6 +275,19 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -284,7 +303,7 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -297,8 +316,6 @@
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -318,7 +335,7 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -331,8 +348,6 @@
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -352,7 +367,7 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -365,8 +380,6 @@
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -386,7 +399,7 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -399,8 +412,6 @@
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -420,7 +431,7 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -433,8 +444,6 @@
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -454,10 +463,8 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
         <right style="medium">
           <color rgb="FFCCCCCC"/>
         </right>
@@ -467,13 +474,11 @@
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -488,7 +493,7 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right style="medium">
           <color rgb="FFCCCCCC"/>
@@ -499,8 +504,6 @@
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -508,6 +511,34 @@
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -524,8 +555,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Таблица1" displayName="Таблица1" ref="A1:H5" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" tableBorderDxfId="9">
-  <autoFilter ref="A1:H5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Таблица1" displayName="Таблица1" ref="A1:H6" totalsRowShown="0" headerRowDxfId="10" dataDxfId="0" tableBorderDxfId="9">
+  <autoFilter ref="A1:H6"/>
   <tableColumns count="8">
     <tableColumn id="1" name="ID" dataDxfId="8"/>
     <tableColumn id="2" name="Название" dataDxfId="7"/>
@@ -534,7 +565,7 @@
     <tableColumn id="5" name="Шаги" dataDxfId="4"/>
     <tableColumn id="6" name="Ожидаемый результат" dataDxfId="3"/>
     <tableColumn id="7" name="Комментарий" dataDxfId="2"/>
-    <tableColumn id="8" name="Статус"/>
+    <tableColumn id="8" name="Статус" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -803,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.5703125" customWidth="1"/>
@@ -816,37 +847,37 @@
     <col min="8" max="8" width="9.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="101.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:25" ht="101.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="9" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -864,11 +895,11 @@
       <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="101.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:25" ht="101.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
@@ -890,11 +921,11 @@
       <c r="G3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="101.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:25" ht="101.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>10</v>
       </c>
@@ -916,11 +947,11 @@
       <c r="G4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="115.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:25" ht="115.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>14</v>
       </c>
@@ -942,9 +973,55 @@
       <c r="G5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="8" t="s">
         <v>26</v>
       </c>
+    </row>
+    <row r="6" spans="1:25" ht="101.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+      <c r="X6" s="5"/>
+      <c r="Y6" s="5"/>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="H12" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>